<commit_message>
aplitivo mobile para notificações
</commit_message>
<xml_diff>
--- a/novasFuncionalidades.xlsx
+++ b/novasFuncionalidades.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Particular\Documents\AutorizaSekitaF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Particular\Desktop\TI_software\Projetos\AutorizaSekita\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6D058A1-5C82-4E47-B1B5-B49A19B77346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26AA28E-2427-4316-B4D7-6E611EF17135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>Numero</t>
   </si>
@@ -70,14 +70,28 @@
   </si>
   <si>
     <t>Disparar alertas entre convocações.</t>
+  </si>
+  <si>
+    <t>Requisições de compra</t>
+  </si>
+  <si>
+    <t>Aumento de salario: supervisor encaminha solicitação com os dados para o diretor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -126,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -136,6 +150,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,13 +434,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:D11"/>
+  <dimension ref="A2:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="72" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="75.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -433,7 +452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
         <v>1</v>
@@ -441,8 +460,11 @@
       <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
         <v>5</v>
@@ -451,7 +473,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -459,49 +481,59 @@
       <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" s="2"/>
       <c r="C8" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="2"/>
       <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
       <c r="C10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
       <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+      <c r="C12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>